<commit_message>
Fixing error in Excel file
</commit_message>
<xml_diff>
--- a/manual/Ebola cases imported into Europe.xlsx
+++ b/manual/Ebola cases imported into Europe.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/nick/Documents/Ebola/ebola-importation/manual/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BFE7F417-21CE-354B-B357-ADEDAA376EF8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B76617B5-66FB-5A42-A808-A640F7E25608}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="760" windowWidth="34560" windowHeight="21580" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -16,7 +16,20 @@
     <sheet name="Data" sheetId="1" r:id="rId1"/>
     <sheet name="Dictionary" sheetId="2" r:id="rId2"/>
   </sheets>
-  <calcPr calcId="0"/>
+  <calcPr calcId="191029"/>
+  <extLst>
+    <ext xmlns:xcalcf="http://schemas.microsoft.com/office/spreadsheetml/2018/calcfeatures" uri="{B58B0392-4F1F-4190-BB64-5DF3571DCE5F}">
+      <xcalcf:calcFeatures>
+        <xcalcf:feature name="microsoft.com:RD"/>
+        <xcalcf:feature name="microsoft.com:Single"/>
+        <xcalcf:feature name="microsoft.com:FV"/>
+        <xcalcf:feature name="microsoft.com:CNMTM"/>
+        <xcalcf:feature name="microsoft.com:LET_WF"/>
+        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
+        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
+      </xcalcf:calcFeatures>
+    </ext>
+  </extLst>
 </workbook>
 </file>
 
@@ -39,7 +52,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="986" uniqueCount="345">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="1146" uniqueCount="441">
   <si>
     <t>Manual</t>
   </si>
@@ -1228,6 +1241,294 @@
   <si>
     <t>lab tech (Porton Down)</t>
   </si>
+  <si>
+    <t>https://www.thelancet.com/journals/lanres/article/PIIS2213-2600(15)00180-0/fulltext</t>
+  </si>
+  <si>
+    <t>22 Aug 2014</t>
+  </si>
+  <si>
+    <t>24 Aug 2014</t>
+  </si>
+  <si>
+    <t>3 Sep 2014</t>
+  </si>
+  <si>
+    <t>25 Dec 2014</t>
+  </si>
+  <si>
+    <t>28 Dec 2014</t>
+  </si>
+  <si>
+    <t>29 Dec 2014</t>
+  </si>
+  <si>
+    <t>24 Jan 2015</t>
+  </si>
+  <si>
+    <t>11 Mar 2015</t>
+  </si>
+  <si>
+    <t>12 Mar 2015</t>
+  </si>
+  <si>
+    <t>27 Mar 2015</t>
+  </si>
+  <si>
+    <t>3 Dec 2014</t>
+  </si>
+  <si>
+    <t>6 Dec 2014</t>
+  </si>
+  <si>
+    <t>22 Dec 2014</t>
+  </si>
+  <si>
+    <t>12 Aug 2014</t>
+  </si>
+  <si>
+    <t>1 Aug 2014</t>
+  </si>
+  <si>
+    <t>5 Aug 2014</t>
+  </si>
+  <si>
+    <t>6 Aug 2014</t>
+  </si>
+  <si>
+    <t>7 Aug 2014</t>
+  </si>
+  <si>
+    <t>25 Sep 2014</t>
+  </si>
+  <si>
+    <t>21 Sep 2014</t>
+  </si>
+  <si>
+    <t>22 Sep 2014</t>
+  </si>
+  <si>
+    <t>30 Sep 2014</t>
+  </si>
+  <si>
+    <t>6 Oct 2014</t>
+  </si>
+  <si>
+    <t>5 Nov 2014</t>
+  </si>
+  <si>
+    <t>16 Nov 2014</t>
+  </si>
+  <si>
+    <t>17 Nov 2014</t>
+  </si>
+  <si>
+    <t>20 Nov 2014</t>
+  </si>
+  <si>
+    <t>21 Nov 2014</t>
+  </si>
+  <si>
+    <t>24 Nov 2014</t>
+  </si>
+  <si>
+    <t>25 Nov 2014</t>
+  </si>
+  <si>
+    <t>2 Jan 2015</t>
+  </si>
+  <si>
+    <t>18 May 2026</t>
+  </si>
+  <si>
+    <t>20 May 2026</t>
+  </si>
+  <si>
+    <t>6 Jun 2026</t>
+  </si>
+  <si>
+    <t>14 Oct 2014</t>
+  </si>
+  <si>
+    <t>8 Oct 2014</t>
+  </si>
+  <si>
+    <t>9 Oct 2014</t>
+  </si>
+  <si>
+    <t>3 Oct 2014</t>
+  </si>
+  <si>
+    <t>19 Nov 2014</t>
+  </si>
+  <si>
+    <t>18 Aug 2014</t>
+  </si>
+  <si>
+    <t>23 Aug 2014</t>
+  </si>
+  <si>
+    <t>27 Aug 2014</t>
+  </si>
+  <si>
+    <t>26 Sep 2014</t>
+  </si>
+  <si>
+    <t>4 Oct 2014</t>
+  </si>
+  <si>
+    <t>5 Oct 2014</t>
+  </si>
+  <si>
+    <t>7 Oct 2014</t>
+  </si>
+  <si>
+    <t>20 Oct 2014</t>
+  </si>
+  <si>
+    <t>1 Nov 2014</t>
+  </si>
+  <si>
+    <t>23 Nov 2014</t>
+  </si>
+  <si>
+    <t>23 Jul 2014</t>
+  </si>
+  <si>
+    <t>27 Jul 2014</t>
+  </si>
+  <si>
+    <t>2 Aug 2014</t>
+  </si>
+  <si>
+    <t>21 Aug 2014</t>
+  </si>
+  <si>
+    <t>22 Jul 2014</t>
+  </si>
+  <si>
+    <t>26 Jul 2014</t>
+  </si>
+  <si>
+    <t>4 Aug 2014</t>
+  </si>
+  <si>
+    <t>19 Aug 2014</t>
+  </si>
+  <si>
+    <t>29 Aug 2014</t>
+  </si>
+  <si>
+    <t>1 Sep 2014</t>
+  </si>
+  <si>
+    <t>4 Sep 2014</t>
+  </si>
+  <si>
+    <t>5 Sep 2014</t>
+  </si>
+  <si>
+    <t>6 Sep 2014</t>
+  </si>
+  <si>
+    <t>7 Sep 2014</t>
+  </si>
+  <si>
+    <t>9 Sep 2014</t>
+  </si>
+  <si>
+    <t>19 Oct 2014</t>
+  </si>
+  <si>
+    <t>11 Oct 2014</t>
+  </si>
+  <si>
+    <t>24 Oct 2014</t>
+  </si>
+  <si>
+    <t>15 Oct 2014</t>
+  </si>
+  <si>
+    <t>28 Oct 2014</t>
+  </si>
+  <si>
+    <t>1 Oct 2014</t>
+  </si>
+  <si>
+    <t>2 Oct 2014</t>
+  </si>
+  <si>
+    <t>22 Oct 2014</t>
+  </si>
+  <si>
+    <t>23 Oct 2014</t>
+  </si>
+  <si>
+    <t>11 Nov 2014</t>
+  </si>
+  <si>
+    <t>6 Nov 2014</t>
+  </si>
+  <si>
+    <t>15 Nov 2014</t>
+  </si>
+  <si>
+    <t>10 Nov 2014</t>
+  </si>
+  <si>
+    <t>13 Mar 2015</t>
+  </si>
+  <si>
+    <t>9 Apr 2015</t>
+  </si>
+  <si>
+    <t>5 Nov 1976</t>
+  </si>
+  <si>
+    <t>11 Nov 1976</t>
+  </si>
+  <si>
+    <t>12 Nov 1976</t>
+  </si>
+  <si>
+    <t>25 Feb 1977</t>
+  </si>
+  <si>
+    <t>16 Nov 1994</t>
+  </si>
+  <si>
+    <t>24 Nov 1994</t>
+  </si>
+  <si>
+    <t>26 Nov 1994</t>
+  </si>
+  <si>
+    <t>30 Nov 1994</t>
+  </si>
+  <si>
+    <t>1 Dec 1994</t>
+  </si>
+  <si>
+    <t>8 Dec 1994</t>
+  </si>
+  <si>
+    <t>10 May 2015</t>
+  </si>
+  <si>
+    <t>11 May 2015</t>
+  </si>
+  <si>
+    <t>12 May 2015</t>
+  </si>
+  <si>
+    <t>7 May 2015</t>
+  </si>
+  <si>
+    <t>9 May 2015</t>
+  </si>
+  <si>
+    <t>10 Jun 2015</t>
+  </si>
 </sst>
 </file>
 
@@ -1237,7 +1538,7 @@
     <numFmt numFmtId="164" formatCode="d&quot; &quot;mmm&quot; &quot;yyyy"/>
     <numFmt numFmtId="165" formatCode="d\ mmm\ yyyy"/>
   </numFmts>
-  <fonts count="12" x14ac:knownFonts="1">
+  <fonts count="13" x14ac:knownFonts="1">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -1320,6 +1621,14 @@
       <name val="Arial"/>
       <family val="2"/>
     </font>
+    <font>
+      <u/>
+      <sz val="10"/>
+      <color theme="10"/>
+      <name val="Arial"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
   </fonts>
   <fills count="2">
     <fill>
@@ -1338,10 +1647,11 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="16">
+  <cellXfs count="21">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1"/>
@@ -1372,8 +1682,18 @@
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="165" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="49" fontId="6" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="right" vertical="top"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
+    <xf numFmtId="49" fontId="2" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Hyperlink" xfId="1" builtinId="8"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -1610,7 +1930,7 @@
   <sheetPr>
     <outlinePr summaryBelow="0" summaryRight="0"/>
   </sheetPr>
-  <dimension ref="A1:AZ47"/>
+  <dimension ref="A1:AZ67"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="12.6640625" defaultRowHeight="15.75" customHeight="1" x14ac:dyDescent="0.15"/>
   <cols>
     <col min="1" max="1" width="6.83203125" customWidth="1"/>
@@ -1622,7 +1942,7 @@
     <col min="9" max="9" width="15" customWidth="1"/>
     <col min="10" max="10" width="13.6640625" customWidth="1"/>
     <col min="11" max="11" width="7.1640625" customWidth="1"/>
-    <col min="12" max="12" width="4.6640625" customWidth="1"/>
+    <col min="12" max="12" width="5.6640625" customWidth="1"/>
     <col min="13" max="13" width="35.1640625" customWidth="1"/>
     <col min="14" max="14" width="44.1640625" customWidth="1"/>
     <col min="15" max="15" width="9.5" customWidth="1"/>
@@ -1634,9 +1954,9 @@
     <col min="21" max="21" width="27.1640625" customWidth="1"/>
     <col min="22" max="22" width="13.83203125" customWidth="1"/>
     <col min="23" max="23" width="5" customWidth="1"/>
-    <col min="24" max="24" width="10.1640625" customWidth="1"/>
+    <col min="24" max="24" width="11.6640625" customWidth="1"/>
     <col min="25" max="25" width="12.6640625" customWidth="1"/>
-    <col min="26" max="26" width="10.6640625" customWidth="1"/>
+    <col min="26" max="26" width="11.83203125" customWidth="1"/>
     <col min="27" max="27" width="13.6640625" customWidth="1"/>
     <col min="28" max="28" width="13.5" customWidth="1"/>
     <col min="29" max="29" width="15.1640625" customWidth="1"/>
@@ -1859,32 +2179,32 @@
       <c r="W2" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X2" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y2" s="3" t="s">
+      <c r="X2" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y2" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z2" s="4">
-        <v>41873</v>
-      </c>
-      <c r="AA2" s="4">
-        <v>41875</v>
-      </c>
-      <c r="AB2" s="4">
-        <v>41873</v>
-      </c>
-      <c r="AC2" s="4">
-        <v>41873</v>
-      </c>
-      <c r="AD2" s="4">
-        <v>41875</v>
-      </c>
-      <c r="AE2" s="4">
-        <v>41875</v>
-      </c>
-      <c r="AF2" s="4">
-        <v>41885</v>
+      <c r="Z2" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="AA2" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="AB2" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="AC2" s="17" t="s">
+        <v>346</v>
+      </c>
+      <c r="AD2" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="AE2" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="AF2" s="17" t="s">
+        <v>348</v>
       </c>
       <c r="AG2" s="2" t="s">
         <v>53</v>
@@ -1989,32 +2309,32 @@
       <c r="W3" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X3" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y3" s="4">
-        <v>41998</v>
-      </c>
-      <c r="Z3" s="4">
-        <v>42001</v>
-      </c>
-      <c r="AA3" s="4">
-        <v>42002</v>
-      </c>
-      <c r="AB3" s="4">
-        <v>42002</v>
-      </c>
-      <c r="AC3" s="4">
-        <v>42002</v>
-      </c>
-      <c r="AD3" s="4">
-        <v>42001</v>
-      </c>
-      <c r="AE3" s="4">
-        <v>42001</v>
-      </c>
-      <c r="AF3" s="4">
-        <v>42028</v>
+      <c r="X3" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y3" s="17" t="s">
+        <v>349</v>
+      </c>
+      <c r="Z3" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="AA3" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="AB3" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="AC3" s="17" t="s">
+        <v>351</v>
+      </c>
+      <c r="AD3" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="AE3" s="17" t="s">
+        <v>350</v>
+      </c>
+      <c r="AF3" s="17" t="s">
+        <v>352</v>
       </c>
       <c r="AG3" s="2" t="s">
         <v>53</v>
@@ -2125,32 +2445,32 @@
       <c r="W4" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X4" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y4" s="4" t="s">
+      <c r="X4" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y4" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z4" s="4" t="s">
+      <c r="Z4" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA4" s="4">
-        <v>42074</v>
-      </c>
-      <c r="AB4" s="4">
-        <v>42074</v>
-      </c>
-      <c r="AC4" s="4">
-        <v>42074</v>
-      </c>
-      <c r="AD4" s="4">
-        <v>42075</v>
-      </c>
-      <c r="AE4" s="4">
-        <v>42075</v>
-      </c>
-      <c r="AF4" s="4">
-        <v>42090</v>
+      <c r="AA4" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="AB4" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="AC4" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="AD4" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="AE4" s="17" t="s">
+        <v>354</v>
+      </c>
+      <c r="AF4" s="17" t="s">
+        <v>355</v>
       </c>
       <c r="AG4" s="2" t="s">
         <v>53</v>
@@ -2257,32 +2577,32 @@
       <c r="W5" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X5" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y5" s="3" t="s">
+      <c r="X5" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z5" s="3" t="s">
+      <c r="Z5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA5" s="3" t="s">
+      <c r="AA5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB5" s="4">
-        <v>41976</v>
-      </c>
-      <c r="AC5" s="3" t="s">
+      <c r="AB5" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="AC5" s="17" t="s">
+        <v>356</v>
+      </c>
+      <c r="AD5" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AD5" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE5" s="8">
-        <v>41979</v>
-      </c>
-      <c r="AF5" s="4">
-        <v>41995</v>
+      <c r="AE5" s="17" t="s">
+        <v>357</v>
+      </c>
+      <c r="AF5" s="17" t="s">
+        <v>358</v>
       </c>
       <c r="AG5" s="2" t="s">
         <v>53</v>
@@ -2389,31 +2709,31 @@
       <c r="W6" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X6" s="4">
-        <v>41863</v>
-      </c>
-      <c r="Y6" s="4" t="s">
+      <c r="X6" s="17" t="s">
+        <v>359</v>
+      </c>
+      <c r="Y6" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z6" s="4" t="s">
+      <c r="Z6" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA6" s="8">
-        <v>41852</v>
-      </c>
-      <c r="AB6" s="4">
-        <v>41856</v>
-      </c>
-      <c r="AC6" s="4">
-        <v>41856</v>
-      </c>
-      <c r="AD6" s="4">
-        <v>41857</v>
-      </c>
-      <c r="AE6" s="4">
-        <v>41858</v>
-      </c>
-      <c r="AF6" s="3" t="s">
+      <c r="AA6" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="AB6" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="AC6" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="AD6" s="17" t="s">
+        <v>362</v>
+      </c>
+      <c r="AE6" s="17" t="s">
+        <v>363</v>
+      </c>
+      <c r="AF6" s="17" t="s">
         <v>48</v>
       </c>
       <c r="AG6" s="2" t="s">
@@ -2521,31 +2841,31 @@
       <c r="W7" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X7" s="4">
-        <v>41907</v>
-      </c>
-      <c r="Y7" s="4" t="s">
+      <c r="X7" s="17" t="s">
+        <v>364</v>
+      </c>
+      <c r="Y7" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z7" s="4" t="s">
+      <c r="Z7" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA7" s="3" t="s">
+      <c r="AA7" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB7" s="3" t="s">
+      <c r="AB7" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="AC7" s="3" t="s">
+      <c r="AC7" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="AD7" s="9">
-        <v>41903</v>
-      </c>
-      <c r="AE7" s="8">
-        <v>41904</v>
-      </c>
-      <c r="AF7" s="10" t="s">
+      <c r="AD7" s="18" t="s">
+        <v>365</v>
+      </c>
+      <c r="AE7" s="17" t="s">
+        <v>366</v>
+      </c>
+      <c r="AF7" s="18" t="s">
         <v>48</v>
       </c>
       <c r="AG7" s="2" t="s">
@@ -2655,32 +2975,32 @@
       <c r="W8" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y8" s="3" t="s">
+      <c r="X8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y8" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z8" s="4">
-        <v>41912</v>
-      </c>
-      <c r="AA8" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AB8" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AC8" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AD8" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE8" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF8" s="9">
-        <v>41948</v>
+      <c r="Z8" s="17" t="s">
+        <v>367</v>
+      </c>
+      <c r="AA8" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AB8" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AC8" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AD8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE8" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF8" s="18" t="s">
+        <v>369</v>
       </c>
       <c r="AG8" s="2" t="s">
         <v>53</v>
@@ -2697,7 +3017,9 @@
       <c r="AK8" s="5" t="s">
         <v>113</v>
       </c>
-      <c r="AL8" s="2"/>
+      <c r="AL8" s="16" t="s">
+        <v>345</v>
+      </c>
       <c r="AM8" s="2"/>
       <c r="AN8" s="2"/>
       <c r="AO8" s="2"/>
@@ -2783,32 +3105,32 @@
       <c r="W9" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X9" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y9" s="4" t="s">
+      <c r="X9" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y9" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z9" s="4">
-        <v>41959</v>
-      </c>
-      <c r="AA9" s="4">
-        <v>41960</v>
-      </c>
-      <c r="AB9" s="4">
-        <v>41960</v>
-      </c>
-      <c r="AC9" s="4">
-        <v>41960</v>
-      </c>
-      <c r="AD9" s="4">
-        <v>41963</v>
-      </c>
-      <c r="AE9" s="4">
-        <v>41964</v>
-      </c>
-      <c r="AF9" s="4">
-        <v>41979</v>
+      <c r="Z9" s="17" t="s">
+        <v>370</v>
+      </c>
+      <c r="AA9" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="AB9" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="AC9" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="AD9" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="AE9" s="17" t="s">
+        <v>373</v>
+      </c>
+      <c r="AF9" s="17" t="s">
+        <v>357</v>
       </c>
       <c r="AG9" s="2" t="s">
         <v>53</v>
@@ -2846,10 +3168,10 @@
         <v>9</v>
       </c>
       <c r="B10" s="2">
-        <v>34</v>
+        <v>27</v>
       </c>
       <c r="C10" s="2">
-        <v>18</v>
+        <v>14</v>
       </c>
       <c r="D10" s="2" t="s">
         <v>42</v>
@@ -2870,19 +3192,19 @@
         <v>46</v>
       </c>
       <c r="J10" s="2" t="s">
-        <v>125</v>
+        <v>135</v>
       </c>
       <c r="K10" s="3" t="s">
         <v>48</v>
       </c>
       <c r="L10" s="2">
-        <v>2015</v>
+        <v>2014</v>
       </c>
       <c r="M10" s="2" t="s">
-        <v>126</v>
+        <v>136</v>
       </c>
       <c r="N10" s="2" t="s">
-        <v>327</v>
+        <v>331</v>
       </c>
       <c r="O10" s="2" t="s">
         <v>50</v>
@@ -2891,7 +3213,7 @@
         <v>124</v>
       </c>
       <c r="Q10" s="3">
-        <v>37</v>
+        <v>50</v>
       </c>
       <c r="R10" s="2" t="s">
         <v>51</v>
@@ -2900,7 +3222,7 @@
         <v>42</v>
       </c>
       <c r="T10" s="2" t="s">
-        <v>53</v>
+        <v>42</v>
       </c>
       <c r="U10" s="2" t="s">
         <v>127</v>
@@ -2911,32 +3233,32 @@
       <c r="W10" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X10" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y10" s="3" t="s">
+      <c r="X10" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y10" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z10" s="4">
-        <v>41769</v>
-      </c>
-      <c r="AA10" s="4">
-        <v>41770</v>
-      </c>
-      <c r="AB10" s="4">
-        <v>41771</v>
-      </c>
-      <c r="AC10" s="4">
-        <v>41771</v>
-      </c>
-      <c r="AD10" s="4">
-        <v>41766</v>
-      </c>
-      <c r="AE10" s="4">
-        <v>41768</v>
-      </c>
-      <c r="AF10" s="4">
-        <v>41800</v>
+      <c r="Z10" s="17" t="s">
+        <v>372</v>
+      </c>
+      <c r="AA10" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="AB10" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="AC10" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="AD10" s="17" t="s">
+        <v>374</v>
+      </c>
+      <c r="AE10" s="17" t="s">
+        <v>375</v>
+      </c>
+      <c r="AF10" s="17" t="s">
+        <v>376</v>
       </c>
       <c r="AG10" s="2" t="s">
         <v>53</v>
@@ -2945,26 +3267,20 @@
         <v>0</v>
       </c>
       <c r="AI10" s="5" t="s">
-        <v>128</v>
-      </c>
-      <c r="AJ10" s="5" t="s">
-        <v>129</v>
+        <v>137</v>
+      </c>
+      <c r="AJ10" s="6" t="s">
+        <v>138</v>
       </c>
       <c r="AK10" s="6" t="s">
-        <v>130</v>
-      </c>
-      <c r="AL10" s="6" t="s">
-        <v>131</v>
-      </c>
-      <c r="AM10" s="5" t="s">
-        <v>132</v>
-      </c>
-      <c r="AN10" s="5" t="s">
-        <v>133</v>
-      </c>
-      <c r="AO10" s="5" t="s">
-        <v>134</v>
-      </c>
+        <v>139</v>
+      </c>
+      <c r="AL10" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="AM10" s="2"/>
+      <c r="AN10" s="2"/>
+      <c r="AO10" s="2"/>
       <c r="AP10" s="2"/>
       <c r="AQ10" s="2"/>
       <c r="AR10" s="2"/>
@@ -2980,10 +3296,10 @@
         <v>10</v>
       </c>
       <c r="B11" s="2">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="C11" s="2">
-        <v>14</v>
+        <v>18</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>42</v>
@@ -3004,19 +3320,19 @@
         <v>46</v>
       </c>
       <c r="J11" s="2" t="s">
-        <v>135</v>
+        <v>125</v>
       </c>
       <c r="K11" s="3" t="s">
         <v>48</v>
       </c>
       <c r="L11" s="2">
-        <v>2014</v>
+        <v>2015</v>
       </c>
       <c r="M11" s="2" t="s">
-        <v>136</v>
+        <v>126</v>
       </c>
       <c r="N11" s="2" t="s">
-        <v>331</v>
+        <v>327</v>
       </c>
       <c r="O11" s="2" t="s">
         <v>50</v>
@@ -3025,7 +3341,7 @@
         <v>124</v>
       </c>
       <c r="Q11" s="3">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="R11" s="2" t="s">
         <v>51</v>
@@ -3034,7 +3350,7 @@
         <v>42</v>
       </c>
       <c r="T11" s="2" t="s">
-        <v>42</v>
+        <v>53</v>
       </c>
       <c r="U11" s="2" t="s">
         <v>127</v>
@@ -3045,32 +3361,32 @@
       <c r="W11" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X11" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y11" s="3" t="s">
+      <c r="X11" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y11" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z11" s="4">
-        <v>41963</v>
-      </c>
-      <c r="AA11" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AB11" s="4">
-        <v>41967</v>
-      </c>
-      <c r="AC11" s="4">
-        <v>41967</v>
-      </c>
-      <c r="AD11" s="8">
-        <v>41967</v>
-      </c>
-      <c r="AE11" s="4">
-        <v>41968</v>
-      </c>
-      <c r="AF11" s="4">
-        <v>42006</v>
+      <c r="Z11" s="17" t="s">
+        <v>435</v>
+      </c>
+      <c r="AA11" s="17" t="s">
+        <v>436</v>
+      </c>
+      <c r="AB11" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="AC11" s="17" t="s">
+        <v>437</v>
+      </c>
+      <c r="AD11" s="17" t="s">
+        <v>438</v>
+      </c>
+      <c r="AE11" s="17" t="s">
+        <v>439</v>
+      </c>
+      <c r="AF11" s="17" t="s">
+        <v>440</v>
       </c>
       <c r="AG11" s="2" t="s">
         <v>53</v>
@@ -3079,20 +3395,26 @@
         <v>0</v>
       </c>
       <c r="AI11" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="AJ11" s="6" t="s">
-        <v>138</v>
+        <v>128</v>
+      </c>
+      <c r="AJ11" s="5" t="s">
+        <v>129</v>
       </c>
       <c r="AK11" s="6" t="s">
-        <v>139</v>
-      </c>
-      <c r="AL11" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="AM11" s="2"/>
-      <c r="AN11" s="2"/>
-      <c r="AO11" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="AL11" s="6" t="s">
+        <v>131</v>
+      </c>
+      <c r="AM11" s="5" t="s">
+        <v>132</v>
+      </c>
+      <c r="AN11" s="5" t="s">
+        <v>133</v>
+      </c>
+      <c r="AO11" s="5" t="s">
+        <v>134</v>
+      </c>
       <c r="AP11" s="2"/>
       <c r="AQ11" s="2"/>
       <c r="AR11" s="2"/>
@@ -3173,32 +3495,32 @@
       <c r="W12" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X12" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y12" s="4" t="s">
+      <c r="X12" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y12" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z12" s="4" t="s">
+      <c r="Z12" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA12" s="4" t="s">
+      <c r="AA12" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB12" s="4" t="s">
+      <c r="AB12" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="AC12" s="17" t="s">
+        <v>377</v>
+      </c>
+      <c r="AD12" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AC12" s="4">
-        <v>46160</v>
-      </c>
-      <c r="AD12" s="3" t="s">
-        <v>54</v>
-      </c>
-      <c r="AE12" s="4">
-        <v>46162</v>
-      </c>
-      <c r="AF12" s="8">
-        <v>46179</v>
+      <c r="AE12" s="17" t="s">
+        <v>378</v>
+      </c>
+      <c r="AF12" s="17" t="s">
+        <v>379</v>
       </c>
       <c r="AG12" s="2" t="s">
         <v>148</v>
@@ -3301,31 +3623,31 @@
       <c r="W13" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X13" s="4">
-        <v>41926</v>
-      </c>
-      <c r="Y13" s="4" t="s">
+      <c r="X13" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="Y13" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z13" s="4" t="s">
+      <c r="Z13" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA13" s="3" t="s">
+      <c r="AA13" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB13" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AC13" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AD13" s="8">
-        <v>41920</v>
-      </c>
-      <c r="AE13" s="4">
-        <v>41921</v>
-      </c>
-      <c r="AF13" s="3" t="s">
+      <c r="AB13" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AC13" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AD13" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="AE13" s="17" t="s">
+        <v>382</v>
+      </c>
+      <c r="AF13" s="17" t="s">
         <v>48</v>
       </c>
       <c r="AG13" s="2" t="s">
@@ -3427,32 +3749,32 @@
       <c r="W14" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X14" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y14" s="4" t="s">
+      <c r="X14" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y14" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z14" s="4" t="s">
+      <c r="Z14" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="AA14" s="3" t="s">
+      <c r="AA14" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="AB14" s="4" t="s">
+      <c r="AB14" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="AC14" s="4" t="s">
+      <c r="AC14" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="AD14" s="4">
-        <v>41915</v>
-      </c>
-      <c r="AE14" s="4">
-        <v>41915</v>
-      </c>
-      <c r="AF14" s="4">
-        <v>41962</v>
+      <c r="AD14" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="AE14" s="17" t="s">
+        <v>383</v>
+      </c>
+      <c r="AF14" s="17" t="s">
+        <v>384</v>
       </c>
       <c r="AG14" s="2" t="s">
         <v>53</v>
@@ -3553,32 +3875,32 @@
       <c r="W15" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X15" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y15" s="3" t="s">
+      <c r="X15" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y15" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z15" s="4">
-        <v>41869</v>
-      </c>
-      <c r="AA15" s="4">
-        <v>41875</v>
-      </c>
-      <c r="AB15" s="4">
-        <v>41874</v>
-      </c>
-      <c r="AC15" s="4">
-        <v>41874</v>
-      </c>
-      <c r="AD15" s="4">
-        <v>41878</v>
-      </c>
-      <c r="AE15" s="4">
-        <v>41878</v>
-      </c>
-      <c r="AF15" s="4">
-        <v>41908</v>
+      <c r="Z15" s="17" t="s">
+        <v>385</v>
+      </c>
+      <c r="AA15" s="17" t="s">
+        <v>347</v>
+      </c>
+      <c r="AB15" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="AC15" s="17" t="s">
+        <v>386</v>
+      </c>
+      <c r="AD15" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="AE15" s="17" t="s">
+        <v>387</v>
+      </c>
+      <c r="AF15" s="17" t="s">
+        <v>388</v>
       </c>
       <c r="AG15" s="2" t="s">
         <v>53</v>
@@ -3679,32 +4001,32 @@
       <c r="W16" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X16" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y16" s="3" t="s">
+      <c r="X16" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y16" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z16" s="4">
-        <v>41916</v>
-      </c>
-      <c r="AA16" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AB16" s="4">
-        <v>41917</v>
-      </c>
-      <c r="AC16" s="4">
-        <v>41917</v>
-      </c>
-      <c r="AD16" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AE16" s="4">
-        <v>41919</v>
-      </c>
-      <c r="AF16" s="4">
-        <v>41932</v>
+      <c r="Z16" s="17" t="s">
+        <v>389</v>
+      </c>
+      <c r="AA16" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AB16" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="AC16" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="AD16" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AE16" s="17" t="s">
+        <v>391</v>
+      </c>
+      <c r="AF16" s="17" t="s">
+        <v>392</v>
       </c>
       <c r="AG16" s="2" t="s">
         <v>53</v>
@@ -3803,32 +4125,32 @@
       <c r="W17" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X17" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y17" s="3" t="s">
+      <c r="X17" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y17" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z17" s="3" t="s">
+      <c r="Z17" s="17" t="s">
         <v>187</v>
       </c>
-      <c r="AA17" s="3" t="s">
+      <c r="AA17" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB17" s="3" t="s">
+      <c r="AB17" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="AC17" s="3" t="s">
+      <c r="AC17" s="17" t="s">
         <v>188</v>
       </c>
-      <c r="AD17" s="4" t="s">
+      <c r="AD17" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="AE17" s="4" t="s">
+      <c r="AE17" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="AF17" s="4">
-        <v>41916</v>
+      <c r="AF17" s="17" t="s">
+        <v>389</v>
       </c>
       <c r="AG17" s="2" t="s">
         <v>53</v>
@@ -3929,32 +4251,32 @@
       <c r="W18" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X18" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y18" s="3" t="s">
+      <c r="X18" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z18" s="3" t="s">
+      <c r="Z18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA18" s="3" t="s">
+      <c r="AA18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB18" s="3" t="s">
+      <c r="AB18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AC18" s="3" t="s">
+      <c r="AC18" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AD18" s="4">
-        <v>41944</v>
-      </c>
-      <c r="AE18" s="4">
-        <v>41944</v>
-      </c>
-      <c r="AF18" s="4">
-        <v>41966</v>
+      <c r="AD18" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="AE18" s="17" t="s">
+        <v>393</v>
+      </c>
+      <c r="AF18" s="17" t="s">
+        <v>394</v>
       </c>
       <c r="AG18" s="2" t="s">
         <v>53</v>
@@ -4053,32 +4375,32 @@
       <c r="W19" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X19" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y19" s="3" t="s">
+      <c r="X19" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y19" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z19" s="4">
-        <v>41843</v>
-      </c>
-      <c r="AA19" s="3" t="s">
+      <c r="Z19" s="17" t="s">
+        <v>395</v>
+      </c>
+      <c r="AA19" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB19" s="4">
-        <v>41847</v>
-      </c>
-      <c r="AC19" s="4">
-        <v>41847</v>
-      </c>
-      <c r="AD19" s="4">
-        <v>41852</v>
-      </c>
-      <c r="AE19" s="4">
-        <v>41853</v>
-      </c>
-      <c r="AF19" s="4">
-        <v>41872</v>
+      <c r="AB19" s="17" t="s">
+        <v>396</v>
+      </c>
+      <c r="AC19" s="17" t="s">
+        <v>396</v>
+      </c>
+      <c r="AD19" s="17" t="s">
+        <v>360</v>
+      </c>
+      <c r="AE19" s="17" t="s">
+        <v>397</v>
+      </c>
+      <c r="AF19" s="17" t="s">
+        <v>398</v>
       </c>
       <c r="AG19" s="2" t="s">
         <v>53</v>
@@ -4185,32 +4507,32 @@
       <c r="W20" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X20" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y20" s="4" t="s">
+      <c r="X20" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y20" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z20" s="4">
-        <v>41842</v>
-      </c>
-      <c r="AA20" s="3" t="s">
+      <c r="Z20" s="17" t="s">
+        <v>399</v>
+      </c>
+      <c r="AA20" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB20" s="4">
-        <v>41846</v>
-      </c>
-      <c r="AC20" s="4">
-        <v>41846</v>
-      </c>
-      <c r="AD20" s="4">
-        <v>41855</v>
-      </c>
-      <c r="AE20" s="4">
-        <v>41856</v>
-      </c>
-      <c r="AF20" s="4">
-        <v>41870</v>
+      <c r="AB20" s="17" t="s">
+        <v>400</v>
+      </c>
+      <c r="AC20" s="17" t="s">
+        <v>400</v>
+      </c>
+      <c r="AD20" s="17" t="s">
+        <v>401</v>
+      </c>
+      <c r="AE20" s="17" t="s">
+        <v>361</v>
+      </c>
+      <c r="AF20" s="17" t="s">
+        <v>402</v>
       </c>
       <c r="AG20" s="2" t="s">
         <v>53</v>
@@ -4315,32 +4637,32 @@
       <c r="W21" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X21" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y21" s="4" t="s">
+      <c r="X21" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y21" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z21" s="4">
-        <v>41880</v>
-      </c>
-      <c r="AA21" s="4">
-        <v>41883</v>
-      </c>
-      <c r="AB21" s="4">
-        <v>41883</v>
-      </c>
-      <c r="AC21" s="4">
-        <v>41883</v>
-      </c>
-      <c r="AD21" s="4">
-        <v>41886</v>
-      </c>
-      <c r="AE21" s="4">
-        <v>41887</v>
-      </c>
-      <c r="AF21" s="4">
-        <v>41907</v>
+      <c r="Z21" s="17" t="s">
+        <v>403</v>
+      </c>
+      <c r="AA21" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="AB21" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="AC21" s="17" t="s">
+        <v>404</v>
+      </c>
+      <c r="AD21" s="17" t="s">
+        <v>405</v>
+      </c>
+      <c r="AE21" s="17" t="s">
+        <v>406</v>
+      </c>
+      <c r="AF21" s="17" t="s">
+        <v>364</v>
       </c>
       <c r="AG21" s="2" t="s">
         <v>53</v>
@@ -4447,32 +4769,32 @@
       <c r="W22" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X22" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y22" s="3" t="s">
+      <c r="X22" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y22" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z22" s="4">
-        <v>41888</v>
-      </c>
-      <c r="AA22" s="4">
-        <v>41888</v>
-      </c>
-      <c r="AB22" s="4">
-        <v>41889</v>
-      </c>
-      <c r="AC22" s="4">
-        <v>41889</v>
-      </c>
-      <c r="AD22" s="13" t="s">
+      <c r="Z22" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="AA22" s="17" t="s">
+        <v>407</v>
+      </c>
+      <c r="AB22" s="17" t="s">
+        <v>408</v>
+      </c>
+      <c r="AC22" s="17" t="s">
+        <v>408</v>
+      </c>
+      <c r="AD22" s="19" t="s">
         <v>54</v>
       </c>
-      <c r="AE22" s="4">
-        <v>41891</v>
-      </c>
-      <c r="AF22" s="4">
-        <v>41931</v>
+      <c r="AE22" s="17" t="s">
+        <v>409</v>
+      </c>
+      <c r="AF22" s="17" t="s">
+        <v>410</v>
       </c>
       <c r="AG22" s="2" t="s">
         <v>53</v>
@@ -4573,31 +4895,31 @@
       <c r="W23" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X23" s="4">
-        <v>41920</v>
-      </c>
-      <c r="Y23" s="4" t="s">
+      <c r="X23" s="17" t="s">
+        <v>381</v>
+      </c>
+      <c r="Y23" s="17" t="s">
         <v>219</v>
       </c>
-      <c r="Z23" s="4" t="s">
+      <c r="Z23" s="17" t="s">
         <v>220</v>
       </c>
-      <c r="AA23" s="3" t="s">
+      <c r="AA23" s="17" t="s">
         <v>164</v>
       </c>
-      <c r="AB23" s="4" t="s">
+      <c r="AB23" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="AC23" s="4" t="s">
+      <c r="AC23" s="17" t="s">
         <v>221</v>
       </c>
-      <c r="AD23" s="3" t="s">
+      <c r="AD23" s="17" t="s">
         <v>189</v>
       </c>
-      <c r="AE23" s="3" t="s">
+      <c r="AE23" s="17" t="s">
         <v>101</v>
       </c>
-      <c r="AF23" s="3" t="s">
+      <c r="AF23" s="17" t="s">
         <v>48</v>
       </c>
       <c r="AG23" s="2" t="s">
@@ -4699,32 +5021,32 @@
       <c r="W24" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X24" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y24" s="3" t="s">
+      <c r="X24" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y24" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z24" s="8">
-        <v>41923</v>
-      </c>
-      <c r="AA24" s="4">
-        <v>41923</v>
-      </c>
-      <c r="AB24" s="4">
-        <v>41923</v>
-      </c>
-      <c r="AC24" s="4">
-        <v>41923</v>
-      </c>
-      <c r="AD24" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE24" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF24" s="4">
-        <v>41936</v>
+      <c r="Z24" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="AA24" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="AB24" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="AC24" s="17" t="s">
+        <v>411</v>
+      </c>
+      <c r="AD24" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE24" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF24" s="17" t="s">
+        <v>412</v>
       </c>
       <c r="AG24" s="2" t="s">
         <v>53</v>
@@ -4827,32 +5149,32 @@
       <c r="W25" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X25" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y25" s="3" t="s">
+      <c r="X25" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y25" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z25" s="4">
-        <v>41926</v>
-      </c>
-      <c r="AA25" s="4">
-        <v>41926</v>
-      </c>
-      <c r="AB25" s="4">
-        <v>41927</v>
-      </c>
-      <c r="AC25" s="4">
-        <v>41927</v>
-      </c>
-      <c r="AD25" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE25" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF25" s="4">
-        <v>41940</v>
+      <c r="Z25" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="AA25" s="17" t="s">
+        <v>380</v>
+      </c>
+      <c r="AB25" s="17" t="s">
+        <v>413</v>
+      </c>
+      <c r="AC25" s="17" t="s">
+        <v>413</v>
+      </c>
+      <c r="AD25" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE25" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF25" s="17" t="s">
+        <v>414</v>
       </c>
       <c r="AG25" s="2" t="s">
         <v>53</v>
@@ -4953,32 +5275,32 @@
       <c r="W26" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X26" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y26" s="3" t="s">
+      <c r="X26" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y26" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z26" s="4">
-        <v>41913</v>
-      </c>
-      <c r="AA26" s="4">
-        <v>41914</v>
-      </c>
-      <c r="AB26" s="4">
-        <v>41914</v>
-      </c>
-      <c r="AC26" s="4">
-        <v>41914</v>
-      </c>
-      <c r="AD26" s="4">
-        <v>41917</v>
-      </c>
-      <c r="AE26" s="4">
-        <v>41918</v>
-      </c>
-      <c r="AF26" s="4">
-        <v>41934</v>
+      <c r="Z26" s="17" t="s">
+        <v>415</v>
+      </c>
+      <c r="AA26" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="AB26" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="AC26" s="17" t="s">
+        <v>416</v>
+      </c>
+      <c r="AD26" s="17" t="s">
+        <v>390</v>
+      </c>
+      <c r="AE26" s="17" t="s">
+        <v>368</v>
+      </c>
+      <c r="AF26" s="17" t="s">
+        <v>417</v>
       </c>
       <c r="AG26" s="2" t="s">
         <v>53</v>
@@ -5081,32 +5403,32 @@
       <c r="W27" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X27" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y27" s="4" t="s">
+      <c r="X27" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y27" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z27" s="4">
-        <v>41935</v>
-      </c>
-      <c r="AA27" s="4">
-        <v>41935</v>
-      </c>
-      <c r="AB27" s="4">
-        <v>41935</v>
-      </c>
-      <c r="AC27" s="4">
-        <v>41935</v>
-      </c>
-      <c r="AD27" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE27" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF27" s="4">
-        <v>41954</v>
+      <c r="Z27" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="AA27" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="AB27" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="AC27" s="17" t="s">
+        <v>418</v>
+      </c>
+      <c r="AD27" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE27" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF27" s="17" t="s">
+        <v>419</v>
       </c>
       <c r="AG27" s="2" t="s">
         <v>53</v>
@@ -5209,31 +5531,31 @@
       <c r="W28" s="2" t="s">
         <v>42</v>
       </c>
-      <c r="X28" s="4">
-        <v>41960</v>
-      </c>
-      <c r="Y28" s="3" t="s">
+      <c r="X28" s="17" t="s">
+        <v>371</v>
+      </c>
+      <c r="Y28" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z28" s="4">
-        <v>41949</v>
-      </c>
-      <c r="AA28" s="4">
-        <v>41958</v>
-      </c>
-      <c r="AB28" s="4">
-        <v>41953</v>
-      </c>
-      <c r="AC28" s="4">
-        <v>41953</v>
-      </c>
-      <c r="AD28" s="14">
-        <v>41958</v>
-      </c>
-      <c r="AE28" s="4">
-        <v>41958</v>
-      </c>
-      <c r="AF28" s="3" t="s">
+      <c r="Z28" s="17" t="s">
+        <v>420</v>
+      </c>
+      <c r="AA28" s="17" t="s">
+        <v>421</v>
+      </c>
+      <c r="AB28" s="17" t="s">
+        <v>422</v>
+      </c>
+      <c r="AC28" s="17" t="s">
+        <v>422</v>
+      </c>
+      <c r="AD28" s="19" t="s">
+        <v>421</v>
+      </c>
+      <c r="AE28" s="17" t="s">
+        <v>421</v>
+      </c>
+      <c r="AF28" s="17" t="s">
         <v>48</v>
       </c>
       <c r="AG28" s="2" t="s">
@@ -5337,32 +5659,32 @@
       <c r="W29" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X29" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y29" s="3" t="s">
+      <c r="X29" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y29" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="Z29" s="3" t="s">
+      <c r="Z29" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AA29" s="3" t="s">
+      <c r="AA29" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AB29" s="4">
-        <v>42074</v>
-      </c>
-      <c r="AC29" s="4">
-        <v>42074</v>
-      </c>
-      <c r="AD29" s="4">
-        <v>42076</v>
-      </c>
-      <c r="AE29" s="4">
-        <v>42076</v>
-      </c>
-      <c r="AF29" s="4">
-        <v>42103</v>
+      <c r="AB29" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="AC29" s="17" t="s">
+        <v>353</v>
+      </c>
+      <c r="AD29" s="17" t="s">
+        <v>423</v>
+      </c>
+      <c r="AE29" s="17" t="s">
+        <v>423</v>
+      </c>
+      <c r="AF29" s="17" t="s">
+        <v>424</v>
       </c>
       <c r="AG29" s="2" t="s">
         <v>53</v>
@@ -5411,15 +5733,15 @@
       <c r="U30" s="2"/>
       <c r="V30" s="2"/>
       <c r="W30" s="2"/>
-      <c r="X30" s="2"/>
-      <c r="Y30" s="2"/>
-      <c r="Z30" s="2"/>
-      <c r="AA30" s="2"/>
-      <c r="AB30" s="2"/>
-      <c r="AC30" s="2"/>
-      <c r="AD30" s="2"/>
-      <c r="AE30" s="2"/>
-      <c r="AF30" s="2"/>
+      <c r="X30" s="20"/>
+      <c r="Y30" s="20"/>
+      <c r="Z30" s="20"/>
+      <c r="AA30" s="20"/>
+      <c r="AB30" s="20"/>
+      <c r="AC30" s="20"/>
+      <c r="AD30" s="20"/>
+      <c r="AE30" s="20"/>
+      <c r="AF30" s="20"/>
       <c r="AG30" s="2"/>
       <c r="AH30" s="2"/>
       <c r="AI30" s="2"/>
@@ -5458,15 +5780,15 @@
       <c r="U31" s="2"/>
       <c r="V31" s="2"/>
       <c r="W31" s="2"/>
-      <c r="X31" s="2"/>
-      <c r="Y31" s="2"/>
-      <c r="Z31" s="2"/>
-      <c r="AA31" s="2"/>
-      <c r="AB31" s="2"/>
-      <c r="AC31" s="2"/>
-      <c r="AD31" s="2"/>
-      <c r="AE31" s="2"/>
-      <c r="AF31" s="2"/>
+      <c r="X31" s="20"/>
+      <c r="Y31" s="20"/>
+      <c r="Z31" s="20"/>
+      <c r="AA31" s="20"/>
+      <c r="AB31" s="20"/>
+      <c r="AC31" s="20"/>
+      <c r="AD31" s="20"/>
+      <c r="AE31" s="20"/>
+      <c r="AF31" s="20"/>
       <c r="AG31" s="2"/>
       <c r="AH31" s="2"/>
       <c r="AI31" s="2"/>
@@ -5556,32 +5878,32 @@
       <c r="W32" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X32" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y32" s="4">
-        <v>28069</v>
-      </c>
-      <c r="Z32" s="4">
-        <v>28075</v>
-      </c>
-      <c r="AA32" s="4">
-        <v>28069</v>
-      </c>
-      <c r="AB32" s="4">
-        <v>28075</v>
-      </c>
-      <c r="AC32" s="4">
-        <v>28076</v>
-      </c>
-      <c r="AD32" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="AE32" s="3" t="s">
-        <v>48</v>
-      </c>
-      <c r="AF32" s="4">
-        <v>28181</v>
+      <c r="X32" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y32" s="17" t="s">
+        <v>425</v>
+      </c>
+      <c r="Z32" s="17" t="s">
+        <v>426</v>
+      </c>
+      <c r="AA32" s="17" t="s">
+        <v>425</v>
+      </c>
+      <c r="AB32" s="17" t="s">
+        <v>426</v>
+      </c>
+      <c r="AC32" s="17" t="s">
+        <v>427</v>
+      </c>
+      <c r="AD32" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AE32" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="AF32" s="17" t="s">
+        <v>428</v>
       </c>
       <c r="AG32" s="2" t="s">
         <v>53</v>
@@ -5684,32 +6006,32 @@
       <c r="W33" s="2" t="s">
         <v>53</v>
       </c>
-      <c r="X33" s="4" t="s">
-        <v>48</v>
-      </c>
-      <c r="Y33" s="4">
-        <v>34654</v>
-      </c>
-      <c r="Z33" s="4">
-        <v>34662</v>
-      </c>
-      <c r="AA33" s="4">
-        <v>34664</v>
-      </c>
-      <c r="AB33" s="4" t="s">
+      <c r="X33" s="17" t="s">
+        <v>48</v>
+      </c>
+      <c r="Y33" s="17" t="s">
+        <v>429</v>
+      </c>
+      <c r="Z33" s="17" t="s">
+        <v>430</v>
+      </c>
+      <c r="AA33" s="17" t="s">
+        <v>431</v>
+      </c>
+      <c r="AB33" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AC33" s="4" t="s">
+      <c r="AC33" s="17" t="s">
         <v>54</v>
       </c>
-      <c r="AD33" s="4">
-        <v>34668</v>
-      </c>
-      <c r="AE33" s="4">
-        <v>34669</v>
-      </c>
-      <c r="AF33" s="4">
-        <v>34676</v>
+      <c r="AD33" s="17" t="s">
+        <v>432</v>
+      </c>
+      <c r="AE33" s="17" t="s">
+        <v>433</v>
+      </c>
+      <c r="AF33" s="17" t="s">
+        <v>434</v>
       </c>
       <c r="AG33" s="2" t="s">
         <v>53</v>
@@ -5851,6 +6173,15 @@
       </c>
       <c r="H36" s="2"/>
       <c r="I36" s="2"/>
+      <c r="X36" s="4"/>
+      <c r="Y36" s="3"/>
+      <c r="Z36" s="4"/>
+      <c r="AA36" s="4"/>
+      <c r="AB36" s="4"/>
+      <c r="AC36" s="4"/>
+      <c r="AD36" s="4"/>
+      <c r="AE36" s="4"/>
+      <c r="AF36" s="4"/>
     </row>
     <row r="37" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A37" s="3" t="s">
@@ -5876,6 +6207,15 @@
       </c>
       <c r="H37" s="2"/>
       <c r="I37" s="2"/>
+      <c r="X37" s="4"/>
+      <c r="Y37" s="4"/>
+      <c r="Z37" s="4"/>
+      <c r="AA37" s="4"/>
+      <c r="AB37" s="4"/>
+      <c r="AC37" s="4"/>
+      <c r="AD37" s="4"/>
+      <c r="AE37" s="4"/>
+      <c r="AF37" s="4"/>
     </row>
     <row r="38" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A38" s="3" t="s">
@@ -5901,6 +6241,15 @@
       </c>
       <c r="H38" s="2"/>
       <c r="I38" s="2"/>
+      <c r="X38" s="4"/>
+      <c r="Y38" s="4"/>
+      <c r="Z38" s="4"/>
+      <c r="AA38" s="4"/>
+      <c r="AB38" s="4"/>
+      <c r="AC38" s="4"/>
+      <c r="AD38" s="4"/>
+      <c r="AE38" s="4"/>
+      <c r="AF38" s="4"/>
     </row>
     <row r="39" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A39" s="3" t="s">
@@ -5926,6 +6275,15 @@
       </c>
       <c r="H39" s="2"/>
       <c r="I39" s="2"/>
+      <c r="X39" s="4"/>
+      <c r="Y39" s="3"/>
+      <c r="Z39" s="3"/>
+      <c r="AA39" s="3"/>
+      <c r="AB39" s="4"/>
+      <c r="AC39" s="4"/>
+      <c r="AD39" s="3"/>
+      <c r="AE39" s="8"/>
+      <c r="AF39" s="4"/>
     </row>
     <row r="40" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A40" s="3" t="s">
@@ -5951,6 +6309,15 @@
       </c>
       <c r="H40" s="2"/>
       <c r="I40" s="2"/>
+      <c r="X40" s="4"/>
+      <c r="Y40" s="4"/>
+      <c r="Z40" s="4"/>
+      <c r="AA40" s="8"/>
+      <c r="AB40" s="4"/>
+      <c r="AC40" s="4"/>
+      <c r="AD40" s="4"/>
+      <c r="AE40" s="4"/>
+      <c r="AF40" s="3"/>
     </row>
     <row r="41" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="A41" s="2"/>
@@ -5975,15 +6342,15 @@
       <c r="U41" s="2"/>
       <c r="V41" s="2"/>
       <c r="W41" s="2"/>
-      <c r="X41" s="2"/>
-      <c r="Y41" s="2"/>
-      <c r="Z41" s="2"/>
-      <c r="AA41" s="2"/>
-      <c r="AB41" s="2"/>
-      <c r="AC41" s="2"/>
-      <c r="AD41" s="2"/>
-      <c r="AE41" s="2"/>
-      <c r="AF41" s="2"/>
+      <c r="X41" s="4"/>
+      <c r="Y41" s="4"/>
+      <c r="Z41" s="4"/>
+      <c r="AA41" s="3"/>
+      <c r="AB41" s="3"/>
+      <c r="AC41" s="3"/>
+      <c r="AD41" s="9"/>
+      <c r="AE41" s="8"/>
+      <c r="AF41" s="10"/>
       <c r="AG41" s="2"/>
       <c r="AH41" s="2"/>
       <c r="AI41" s="2"/>
@@ -6029,15 +6396,15 @@
       <c r="U42" s="2"/>
       <c r="V42" s="2"/>
       <c r="W42" s="2"/>
-      <c r="X42" s="2"/>
-      <c r="Y42" s="2"/>
-      <c r="Z42" s="2"/>
-      <c r="AA42" s="2"/>
-      <c r="AB42" s="2"/>
-      <c r="AC42" s="2"/>
-      <c r="AD42" s="2"/>
-      <c r="AE42" s="2"/>
-      <c r="AF42" s="2"/>
+      <c r="X42" s="4"/>
+      <c r="Y42" s="3"/>
+      <c r="Z42" s="4"/>
+      <c r="AA42" s="4"/>
+      <c r="AB42" s="4"/>
+      <c r="AC42" s="4"/>
+      <c r="AD42" s="4"/>
+      <c r="AE42" s="3"/>
+      <c r="AF42" s="9"/>
       <c r="AG42" s="2"/>
       <c r="AH42" s="2"/>
       <c r="AI42" s="2"/>
@@ -6087,19 +6454,23 @@
       <c r="U43" s="2"/>
       <c r="V43" s="2"/>
       <c r="W43" s="2"/>
-      <c r="X43" s="2"/>
-      <c r="Y43" s="2"/>
-      <c r="Z43" s="2"/>
-      <c r="AA43" s="2"/>
-      <c r="AB43" s="2"/>
-      <c r="AC43" s="2"/>
-      <c r="AD43" s="2"/>
-      <c r="AE43" s="2"/>
-      <c r="AF43" s="2"/>
+      <c r="X43" s="4"/>
+      <c r="Y43" s="4"/>
+      <c r="Z43" s="4"/>
+      <c r="AA43" s="4"/>
+      <c r="AB43" s="4"/>
+      <c r="AC43" s="4"/>
+      <c r="AD43" s="4"/>
+      <c r="AE43" s="4"/>
+      <c r="AF43" s="4"/>
       <c r="AG43" s="2"/>
       <c r="AH43" s="2"/>
-      <c r="AI43" s="2"/>
-      <c r="AJ43" s="2"/>
+      <c r="AI43" s="5" t="s">
+        <v>288</v>
+      </c>
+      <c r="AJ43" s="5" t="s">
+        <v>289</v>
+      </c>
       <c r="AK43" s="2"/>
       <c r="AL43" s="2"/>
       <c r="AM43" s="2"/>
@@ -6145,15 +6516,15 @@
       <c r="U44" s="2"/>
       <c r="V44" s="2"/>
       <c r="W44" s="2"/>
-      <c r="X44" s="2"/>
-      <c r="Y44" s="2"/>
-      <c r="Z44" s="2"/>
-      <c r="AA44" s="2"/>
-      <c r="AB44" s="2"/>
-      <c r="AC44" s="2"/>
-      <c r="AD44" s="2"/>
-      <c r="AE44" s="2"/>
-      <c r="AF44" s="2"/>
+      <c r="X44" s="4"/>
+      <c r="Y44" s="3"/>
+      <c r="Z44" s="4"/>
+      <c r="AA44" s="4"/>
+      <c r="AB44" s="4"/>
+      <c r="AC44" s="4"/>
+      <c r="AD44" s="4"/>
+      <c r="AE44" s="4"/>
+      <c r="AF44" s="4"/>
       <c r="AG44" s="2"/>
       <c r="AH44" s="2"/>
       <c r="AI44" s="5" t="s">
@@ -6207,15 +6578,15 @@
       <c r="U45" s="2"/>
       <c r="V45" s="2"/>
       <c r="W45" s="2"/>
-      <c r="X45" s="2"/>
-      <c r="Y45" s="2"/>
-      <c r="Z45" s="2"/>
-      <c r="AA45" s="2"/>
-      <c r="AB45" s="2"/>
-      <c r="AC45" s="2"/>
-      <c r="AD45" s="2"/>
-      <c r="AE45" s="2"/>
-      <c r="AF45" s="2"/>
+      <c r="X45" s="4"/>
+      <c r="Y45" s="3"/>
+      <c r="Z45" s="4"/>
+      <c r="AA45" s="3"/>
+      <c r="AB45" s="4"/>
+      <c r="AC45" s="4"/>
+      <c r="AD45" s="8"/>
+      <c r="AE45" s="4"/>
+      <c r="AF45" s="4"/>
       <c r="AG45" s="2"/>
       <c r="AH45" s="2"/>
       <c r="AI45" s="5" t="s">
@@ -6259,23 +6630,17 @@
       <c r="U46" s="2"/>
       <c r="V46" s="2"/>
       <c r="W46" s="2"/>
-      <c r="X46" s="2"/>
-      <c r="Y46" s="2"/>
-      <c r="Z46" s="2"/>
-      <c r="AA46" s="2"/>
-      <c r="AB46" s="2"/>
-      <c r="AC46" s="2"/>
-      <c r="AD46" s="2"/>
-      <c r="AE46" s="2"/>
-      <c r="AF46" s="2"/>
+      <c r="X46" s="4"/>
+      <c r="Y46" s="4"/>
+      <c r="Z46" s="4"/>
+      <c r="AA46" s="4"/>
+      <c r="AB46" s="4"/>
+      <c r="AC46" s="4"/>
+      <c r="AD46" s="3"/>
+      <c r="AE46" s="4"/>
+      <c r="AF46" s="8"/>
       <c r="AG46" s="2"/>
       <c r="AH46" s="2"/>
-      <c r="AI46" s="5" t="s">
-        <v>288</v>
-      </c>
-      <c r="AJ46" s="5" t="s">
-        <v>289</v>
-      </c>
       <c r="AK46" s="2"/>
       <c r="AL46" s="2"/>
       <c r="AM46" s="2"/>
@@ -6293,6 +6658,235 @@
     </row>
     <row r="47" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
       <c r="H47" s="2"/>
+      <c r="X47" s="4"/>
+      <c r="Y47" s="4"/>
+      <c r="Z47" s="4"/>
+      <c r="AA47" s="3"/>
+      <c r="AB47" s="4"/>
+      <c r="AC47" s="4"/>
+      <c r="AD47" s="8"/>
+      <c r="AE47" s="4"/>
+      <c r="AF47" s="3"/>
+    </row>
+    <row r="48" spans="1:50" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X48" s="4"/>
+      <c r="Y48" s="4"/>
+      <c r="Z48" s="4"/>
+      <c r="AA48" s="3"/>
+      <c r="AB48" s="4"/>
+      <c r="AC48" s="4"/>
+      <c r="AD48" s="4"/>
+      <c r="AE48" s="4"/>
+      <c r="AF48" s="4"/>
+    </row>
+    <row r="49" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X49" s="4"/>
+      <c r="Y49" s="3"/>
+      <c r="Z49" s="4"/>
+      <c r="AA49" s="4"/>
+      <c r="AB49" s="4"/>
+      <c r="AC49" s="4"/>
+      <c r="AD49" s="4"/>
+      <c r="AE49" s="4"/>
+      <c r="AF49" s="4"/>
+    </row>
+    <row r="50" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X50" s="4"/>
+      <c r="Y50" s="3"/>
+      <c r="Z50" s="4"/>
+      <c r="AA50" s="4"/>
+      <c r="AB50" s="4"/>
+      <c r="AC50" s="4"/>
+      <c r="AD50" s="4"/>
+      <c r="AE50" s="4"/>
+      <c r="AF50" s="4"/>
+    </row>
+    <row r="51" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X51" s="4"/>
+      <c r="Y51" s="3"/>
+      <c r="Z51" s="3"/>
+      <c r="AA51" s="3"/>
+      <c r="AB51" s="3"/>
+      <c r="AC51" s="3"/>
+      <c r="AD51" s="4"/>
+      <c r="AE51" s="4"/>
+      <c r="AF51" s="4"/>
+    </row>
+    <row r="52" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X52" s="4"/>
+      <c r="Y52" s="3"/>
+      <c r="Z52" s="3"/>
+      <c r="AA52" s="3"/>
+      <c r="AB52" s="3"/>
+      <c r="AC52" s="3"/>
+      <c r="AD52" s="4"/>
+      <c r="AE52" s="4"/>
+      <c r="AF52" s="4"/>
+    </row>
+    <row r="53" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X53" s="4"/>
+      <c r="Y53" s="3"/>
+      <c r="Z53" s="4"/>
+      <c r="AA53" s="3"/>
+      <c r="AB53" s="4"/>
+      <c r="AC53" s="4"/>
+      <c r="AD53" s="4"/>
+      <c r="AE53" s="4"/>
+      <c r="AF53" s="4"/>
+    </row>
+    <row r="54" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X54" s="4"/>
+      <c r="Y54" s="4"/>
+      <c r="Z54" s="4"/>
+      <c r="AA54" s="3"/>
+      <c r="AB54" s="4"/>
+      <c r="AC54" s="4"/>
+      <c r="AD54" s="4"/>
+      <c r="AE54" s="4"/>
+      <c r="AF54" s="4"/>
+    </row>
+    <row r="55" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X55" s="4"/>
+      <c r="Y55" s="4"/>
+      <c r="Z55" s="4"/>
+      <c r="AA55" s="4"/>
+      <c r="AB55" s="4"/>
+      <c r="AC55" s="4"/>
+      <c r="AD55" s="4"/>
+      <c r="AE55" s="4"/>
+      <c r="AF55" s="4"/>
+    </row>
+    <row r="56" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X56" s="4"/>
+      <c r="Y56" s="3"/>
+      <c r="Z56" s="4"/>
+      <c r="AA56" s="4"/>
+      <c r="AB56" s="4"/>
+      <c r="AC56" s="4"/>
+      <c r="AD56" s="13"/>
+      <c r="AE56" s="4"/>
+      <c r="AF56" s="4"/>
+    </row>
+    <row r="57" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X57" s="4"/>
+      <c r="Y57" s="4"/>
+      <c r="Z57" s="4"/>
+      <c r="AA57" s="3"/>
+      <c r="AB57" s="4"/>
+      <c r="AC57" s="4"/>
+      <c r="AD57" s="3"/>
+      <c r="AE57" s="3"/>
+      <c r="AF57" s="3"/>
+    </row>
+    <row r="58" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X58" s="4"/>
+      <c r="Y58" s="3"/>
+      <c r="Z58" s="8"/>
+      <c r="AA58" s="4"/>
+      <c r="AB58" s="4"/>
+      <c r="AC58" s="4"/>
+      <c r="AD58" s="3"/>
+      <c r="AE58" s="3"/>
+      <c r="AF58" s="4"/>
+    </row>
+    <row r="59" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X59" s="4"/>
+      <c r="Y59" s="3"/>
+      <c r="Z59" s="4"/>
+      <c r="AA59" s="4"/>
+      <c r="AB59" s="4"/>
+      <c r="AC59" s="4"/>
+      <c r="AD59" s="3"/>
+      <c r="AE59" s="3"/>
+      <c r="AF59" s="4"/>
+    </row>
+    <row r="60" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X60" s="4"/>
+      <c r="Y60" s="3"/>
+      <c r="Z60" s="4"/>
+      <c r="AA60" s="4"/>
+      <c r="AB60" s="4"/>
+      <c r="AC60" s="4"/>
+      <c r="AD60" s="4"/>
+      <c r="AE60" s="4"/>
+      <c r="AF60" s="4"/>
+    </row>
+    <row r="61" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X61" s="4"/>
+      <c r="Y61" s="4"/>
+      <c r="Z61" s="4"/>
+      <c r="AA61" s="4"/>
+      <c r="AB61" s="4"/>
+      <c r="AC61" s="4"/>
+      <c r="AD61" s="3"/>
+      <c r="AE61" s="3"/>
+      <c r="AF61" s="4"/>
+    </row>
+    <row r="62" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X62" s="4"/>
+      <c r="Y62" s="3"/>
+      <c r="Z62" s="4"/>
+      <c r="AA62" s="4"/>
+      <c r="AB62" s="4"/>
+      <c r="AC62" s="4"/>
+      <c r="AD62" s="14"/>
+      <c r="AE62" s="4"/>
+      <c r="AF62" s="3"/>
+    </row>
+    <row r="63" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X63" s="4"/>
+      <c r="Y63" s="3"/>
+      <c r="Z63" s="3"/>
+      <c r="AA63" s="3"/>
+      <c r="AB63" s="4"/>
+      <c r="AC63" s="4"/>
+      <c r="AD63" s="4"/>
+      <c r="AE63" s="4"/>
+      <c r="AF63" s="4"/>
+    </row>
+    <row r="64" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X64" s="2"/>
+      <c r="Y64" s="2"/>
+      <c r="Z64" s="2"/>
+      <c r="AA64" s="2"/>
+      <c r="AB64" s="2"/>
+      <c r="AC64" s="2"/>
+      <c r="AD64" s="2"/>
+      <c r="AE64" s="2"/>
+      <c r="AF64" s="2"/>
+    </row>
+    <row r="65" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X65" s="2"/>
+      <c r="Y65" s="2"/>
+      <c r="Z65" s="2"/>
+      <c r="AA65" s="2"/>
+      <c r="AB65" s="2"/>
+      <c r="AC65" s="2"/>
+      <c r="AD65" s="2"/>
+      <c r="AE65" s="2"/>
+      <c r="AF65" s="2"/>
+    </row>
+    <row r="66" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X66" s="4"/>
+      <c r="Y66" s="4"/>
+      <c r="Z66" s="4"/>
+      <c r="AA66" s="4"/>
+      <c r="AB66" s="4"/>
+      <c r="AC66" s="4"/>
+      <c r="AD66" s="4"/>
+      <c r="AE66" s="3"/>
+      <c r="AF66" s="4"/>
+    </row>
+    <row r="67" spans="24:32" ht="15.75" customHeight="1" x14ac:dyDescent="0.15">
+      <c r="X67" s="4"/>
+      <c r="Y67" s="4"/>
+      <c r="Z67" s="4"/>
+      <c r="AA67" s="4"/>
+      <c r="AB67" s="4"/>
+      <c r="AC67" s="4"/>
+      <c r="AD67" s="4"/>
+      <c r="AE67" s="4"/>
+      <c r="AF67" s="4"/>
     </row>
   </sheetData>
   <hyperlinks>
@@ -6337,17 +6931,17 @@
     <hyperlink ref="AJ9" r:id="rId39" xr:uid="{00000000-0004-0000-0000-000026000000}"/>
     <hyperlink ref="AK9" r:id="rId40" xr:uid="{00000000-0004-0000-0000-000027000000}"/>
     <hyperlink ref="AL9" r:id="rId41" xr:uid="{00000000-0004-0000-0000-000028000000}"/>
-    <hyperlink ref="AI10" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
-    <hyperlink ref="AJ10" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
-    <hyperlink ref="AK10" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
-    <hyperlink ref="AL10" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
-    <hyperlink ref="AM10" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
-    <hyperlink ref="AN10" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
-    <hyperlink ref="AO10" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
-    <hyperlink ref="AI11" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
-    <hyperlink ref="AJ11" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
-    <hyperlink ref="AK11" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
-    <hyperlink ref="AL11" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
+    <hyperlink ref="AI11" r:id="rId42" xr:uid="{00000000-0004-0000-0000-000029000000}"/>
+    <hyperlink ref="AJ11" r:id="rId43" xr:uid="{00000000-0004-0000-0000-00002A000000}"/>
+    <hyperlink ref="AK11" r:id="rId44" xr:uid="{00000000-0004-0000-0000-00002B000000}"/>
+    <hyperlink ref="AL11" r:id="rId45" xr:uid="{00000000-0004-0000-0000-00002C000000}"/>
+    <hyperlink ref="AM11" r:id="rId46" xr:uid="{00000000-0004-0000-0000-00002D000000}"/>
+    <hyperlink ref="AN11" r:id="rId47" xr:uid="{00000000-0004-0000-0000-00002E000000}"/>
+    <hyperlink ref="AO11" r:id="rId48" xr:uid="{00000000-0004-0000-0000-00002F000000}"/>
+    <hyperlink ref="AI10" r:id="rId49" xr:uid="{00000000-0004-0000-0000-000030000000}"/>
+    <hyperlink ref="AJ10" r:id="rId50" xr:uid="{00000000-0004-0000-0000-000031000000}"/>
+    <hyperlink ref="AK10" r:id="rId51" xr:uid="{00000000-0004-0000-0000-000032000000}"/>
+    <hyperlink ref="AL10" r:id="rId52" xr:uid="{00000000-0004-0000-0000-000033000000}"/>
     <hyperlink ref="AI12" r:id="rId53" location="c34443" xr:uid="{00000000-0004-0000-0000-000034000000}"/>
     <hyperlink ref="AJ12" r:id="rId54" xr:uid="{00000000-0004-0000-0000-000035000000}"/>
     <hyperlink ref="AK12" r:id="rId55" xr:uid="{00000000-0004-0000-0000-000036000000}"/>
@@ -6417,11 +7011,12 @@
     <hyperlink ref="AJ44" r:id="rId119" xr:uid="{00000000-0004-0000-0000-000076000000}"/>
     <hyperlink ref="AI45" r:id="rId120" xr:uid="{00000000-0004-0000-0000-000077000000}"/>
     <hyperlink ref="AJ45" r:id="rId121" xr:uid="{00000000-0004-0000-0000-000078000000}"/>
-    <hyperlink ref="AI46" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
-    <hyperlink ref="AJ46" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="AI43" r:id="rId122" xr:uid="{00000000-0004-0000-0000-000079000000}"/>
+    <hyperlink ref="AJ43" r:id="rId123" xr:uid="{00000000-0004-0000-0000-00007A000000}"/>
+    <hyperlink ref="AL8" r:id="rId124" xr:uid="{7B7EE7A4-BF61-874E-BEFF-9D98AA22AFBD}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <legacyDrawing r:id="rId124"/>
+  <legacyDrawing r:id="rId125"/>
 </worksheet>
 </file>
 

</xml_diff>